<commit_message>
Add International Journal of Music Mediation and current board
</commit_message>
<xml_diff>
--- a/data/xlsx/editorial_histories.xlsx
+++ b/data/xlsx/editorial_histories.xlsx
@@ -491,7 +491,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H227"/>
+  <dimension ref="A1:H246"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -9189,6 +9189,462 @@
         </is>
       </c>
       <c r="H227" t="inlineStr"/>
+    </row>
+    <row r="228" ht="26.399999618530273" hidden="0" customHeight="1">
+      <c r="A228" t="str" s="7">
+        <v>International Journal of Music Mediation (IJMM)</v>
+      </c>
+      <c r="B228" t="str" s="7">
+        <v>Axel Petri-Preis</v>
+      </c>
+      <c r="C228" t="str" s="7">
+        <v>Editor-in-chief</v>
+      </c>
+      <c r="D228" t="str" s="7">
+        <v>present (start date unknown)</v>
+      </c>
+      <c r="E228" t="str" s="7">
+        <v>mdw – University of Music and Performing Arts Vienna</v>
+      </c>
+      <c r="F228" t="str" s="7">
+        <v>High</v>
+      </c>
+      <c r="G228" t="str" s="7">
+        <v>https://ijmm.world/ijmm/about/editorialTeam (verified 2026-10-13)</v>
+      </c>
+      <c r="H228" s="7"/>
+    </row>
+    <row r="229" ht="26.399999618530273" hidden="0" customHeight="1">
+      <c r="A229" t="str" s="7">
+        <v>International Journal of Music Mediation (IJMM)</v>
+      </c>
+      <c r="B229" t="str" s="7">
+        <v>Irina Kirchberg</v>
+      </c>
+      <c r="C229" t="str" s="7">
+        <v>Editor</v>
+      </c>
+      <c r="D229" t="str" s="7">
+        <v>present (start date unknown)</v>
+      </c>
+      <c r="E229" t="str" s="7">
+        <v>University of Montreal / ARTENSO</v>
+      </c>
+      <c r="F229" t="str" s="7">
+        <v>High</v>
+      </c>
+      <c r="G229" t="str" s="7">
+        <v>https://ijmm.world/ijmm/about/editorialTeam (verified 2026-10-13)</v>
+      </c>
+      <c r="H229" s="7"/>
+    </row>
+    <row r="230" ht="26.399999618530273" hidden="0" customHeight="1">
+      <c r="A230" t="str" s="7">
+        <v>International Journal of Music Mediation (IJMM)</v>
+      </c>
+      <c r="B230" t="str" s="7">
+        <v>Irena Müller-Brozovic</v>
+      </c>
+      <c r="C230" t="str" s="7">
+        <v>Editor</v>
+      </c>
+      <c r="D230" t="str" s="7">
+        <v>present (start date unknown)</v>
+      </c>
+      <c r="E230" t="str" s="7">
+        <v>Anton Bruckner Private University / Bern University of Applied Sciences</v>
+      </c>
+      <c r="F230" t="str" s="7">
+        <v>High</v>
+      </c>
+      <c r="G230" t="str" s="7">
+        <v>https://ijmm.world/ijmm/about/editorialTeam (verified 2026-10-13)</v>
+      </c>
+      <c r="H230" s="7"/>
+    </row>
+    <row r="231" ht="26.399999618530273" hidden="0" customHeight="1">
+      <c r="A231" t="str" s="7">
+        <v>International Journal of Music Mediation (IJMM)</v>
+      </c>
+      <c r="B231" t="str" s="7">
+        <v>Viktória Várkonyi</v>
+      </c>
+      <c r="C231" t="str" s="7">
+        <v>Associate Editor</v>
+      </c>
+      <c r="D231" t="str" s="7">
+        <v>present (start date unknown)</v>
+      </c>
+      <c r="E231" t="str" s="7">
+        <v>mdw – University of Music and Performing Arts Vienna</v>
+      </c>
+      <c r="F231" t="str" s="7">
+        <v>High</v>
+      </c>
+      <c r="G231" t="str" s="7">
+        <v>https://ijmm.world/ijmm/about/editorialTeam (verified 2026-10-13)</v>
+      </c>
+      <c r="H231" s="7"/>
+    </row>
+    <row r="232" ht="26.399999618530273" hidden="0" customHeight="1">
+      <c r="A232" t="str" s="7">
+        <v>International Journal of Music Mediation (IJMM)</v>
+      </c>
+      <c r="B232" t="str" s="7">
+        <v>Nadia Thaler</v>
+      </c>
+      <c r="C232" t="str" s="7">
+        <v>Editorial Assistant</v>
+      </c>
+      <c r="D232" t="str" s="7">
+        <v>present (start date unknown)</v>
+      </c>
+      <c r="E232" t="str" s="7">
+        <v>mdw – University of Music and Performing Arts Vienna</v>
+      </c>
+      <c r="F232" t="str" s="7">
+        <v>High</v>
+      </c>
+      <c r="G232" t="str" s="7">
+        <v>https://ijmm.world/ijmm/about/editorialTeam (verified 2026-10-13)</v>
+      </c>
+      <c r="H232" s="7"/>
+    </row>
+    <row r="233" ht="26.399999618530273" hidden="0" customHeight="1">
+      <c r="A233" t="str" s="7">
+        <v>International Journal of Music Mediation (IJMM)</v>
+      </c>
+      <c r="B233" t="str" s="7">
+        <v>Manuel Cañas Escudero</v>
+      </c>
+      <c r="C233" t="str" s="7">
+        <v>Advisory Board member</v>
+      </c>
+      <c r="D233" t="str" s="7">
+        <v>present (start date unknown)</v>
+      </c>
+      <c r="E233" t="str" s="7">
+        <v>Musikene</v>
+      </c>
+      <c r="F233" t="str" s="7">
+        <v>High</v>
+      </c>
+      <c r="G233" t="str" s="7">
+        <v>https://ijmm.world/ijmm/advisory_board (verified 2026-10-13)</v>
+      </c>
+      <c r="H233" s="7"/>
+    </row>
+    <row r="234" ht="26.399999618530273" hidden="0" customHeight="1">
+      <c r="A234" t="str" s="7">
+        <v>International Journal of Music Mediation (IJMM)</v>
+      </c>
+      <c r="B234" t="str" s="7">
+        <v>Sarah Chaker</v>
+      </c>
+      <c r="C234" t="str" s="7">
+        <v>Advisory Board member</v>
+      </c>
+      <c r="D234" t="str" s="7">
+        <v>present (start date unknown)</v>
+      </c>
+      <c r="E234" t="str" s="7">
+        <v>mdw – University of Music and Performing Arts Vienna</v>
+      </c>
+      <c r="F234" t="str" s="7">
+        <v>High</v>
+      </c>
+      <c r="G234" t="str" s="7">
+        <v>https://ijmm.world/ijmm/advisory_board (verified 2026-10-13)</v>
+      </c>
+      <c r="H234" s="7"/>
+    </row>
+    <row r="235" ht="26.399999618530273" hidden="0" customHeight="1">
+      <c r="A235" t="str" s="7">
+        <v>International Journal of Music Mediation (IJMM)</v>
+      </c>
+      <c r="B235" t="str" s="7">
+        <v>Ana Čorić</v>
+      </c>
+      <c r="C235" t="str" s="7">
+        <v>Advisory Board member</v>
+      </c>
+      <c r="D235" t="str" s="7">
+        <v>present (start date unknown)</v>
+      </c>
+      <c r="E235" t="str" s="7">
+        <v>University of Zagreb</v>
+      </c>
+      <c r="F235" t="str" s="7">
+        <v>High</v>
+      </c>
+      <c r="G235" t="str" s="7">
+        <v>https://ijmm.world/ijmm/advisory_board (verified 2026-10-13)</v>
+      </c>
+      <c r="H235" s="7"/>
+    </row>
+    <row r="236" ht="26.399999618530273" hidden="0" customHeight="1">
+      <c r="A236" t="str" s="7">
+        <v>International Journal of Music Mediation (IJMM)</v>
+      </c>
+      <c r="B236" t="str" s="7">
+        <v>Emily Dollman</v>
+      </c>
+      <c r="C236" t="str" s="7">
+        <v>Advisory Board member</v>
+      </c>
+      <c r="D236" t="str" s="7">
+        <v>present (start date unknown)</v>
+      </c>
+      <c r="E236" t="str" s="7">
+        <v>Elder Conservatorium of Music / University of Adelaide</v>
+      </c>
+      <c r="F236" t="str" s="7">
+        <v>High</v>
+      </c>
+      <c r="G236" t="str" s="7">
+        <v>https://ijmm.world/ijmm/advisory_board (verified 2026-10-13)</v>
+      </c>
+      <c r="H236" s="7"/>
+    </row>
+    <row r="237" ht="26.399999618530273" hidden="0" customHeight="1">
+      <c r="A237" t="str" s="7">
+        <v>International Journal of Music Mediation (IJMM)</v>
+      </c>
+      <c r="B237" t="str" s="7">
+        <v>Heloisa Feichas</v>
+      </c>
+      <c r="C237" t="str" s="7">
+        <v>Advisory Board member</v>
+      </c>
+      <c r="D237" t="str" s="7">
+        <v>present (start date unknown)</v>
+      </c>
+      <c r="E237" t="str" s="7">
+        <v>Music School of Federal University of Minas Gerais</v>
+      </c>
+      <c r="F237" t="str" s="7">
+        <v>High</v>
+      </c>
+      <c r="G237" t="str" s="7">
+        <v>https://ijmm.world/ijmm/advisory_board (verified 2026-10-13)</v>
+      </c>
+      <c r="H237" s="7"/>
+    </row>
+    <row r="238" ht="26.399999618530273" hidden="0" customHeight="1">
+      <c r="A238" t="str" s="7">
+        <v>International Journal of Music Mediation (IJMM)</v>
+      </c>
+      <c r="B238" t="str" s="7">
+        <v>Sean Gregory</v>
+      </c>
+      <c r="C238" t="str" s="7">
+        <v>Advisory Board member</v>
+      </c>
+      <c r="D238" t="str" s="7">
+        <v>present (start date unknown)</v>
+      </c>
+      <c r="E238" t="str" s="7">
+        <v>Guildhall School of Music</v>
+      </c>
+      <c r="F238" t="str" s="7">
+        <v>High</v>
+      </c>
+      <c r="G238" t="str" s="7">
+        <v>https://ijmm.world/ijmm/advisory_board (verified 2026-10-13)</v>
+      </c>
+      <c r="H238" s="7"/>
+    </row>
+    <row r="239" ht="26.399999618530273" hidden="0" customHeight="1">
+      <c r="A239" t="str" s="7">
+        <v>International Journal of Music Mediation (IJMM)</v>
+      </c>
+      <c r="B239" t="str" s="7">
+        <v>Lukas Pairon</v>
+      </c>
+      <c r="C239" t="str" s="7">
+        <v>Advisory Board member</v>
+      </c>
+      <c r="D239" t="str" s="7">
+        <v>present (start date unknown)</v>
+      </c>
+      <c r="E239" t="str" s="7">
+        <v>SIMM / CESAMM / Ghent University and University College</v>
+      </c>
+      <c r="F239" t="str" s="7">
+        <v>High</v>
+      </c>
+      <c r="G239" t="str" s="7">
+        <v>https://ijmm.world/ijmm/advisory_board (verified 2026-10-13)</v>
+      </c>
+      <c r="H239" s="7"/>
+    </row>
+    <row r="240" ht="26.399999618530273" hidden="0" customHeight="1">
+      <c r="A240" t="str" s="7">
+        <v>International Journal of Music Mediation (IJMM)</v>
+      </c>
+      <c r="B240" t="str" s="7">
+        <v>Sylvie Pebrier</v>
+      </c>
+      <c r="C240" t="str" s="7">
+        <v>Advisory Board member</v>
+      </c>
+      <c r="D240" t="str" s="7">
+        <v>present (start date unknown)</v>
+      </c>
+      <c r="E240" t="str" s="7">
+        <v>Paris Conservatory / ANICEA</v>
+      </c>
+      <c r="F240" t="str" s="7">
+        <v>High</v>
+      </c>
+      <c r="G240" t="str" s="7">
+        <v>https://ijmm.world/ijmm/advisory_board (verified 2026-10-13)</v>
+      </c>
+      <c r="H240" s="7"/>
+    </row>
+    <row r="241" ht="26.399999618530273" hidden="0" customHeight="1">
+      <c r="A241" t="str" s="7">
+        <v>International Journal of Music Mediation (IJMM)</v>
+      </c>
+      <c r="B241" t="str" s="7">
+        <v>Peter Peters</v>
+      </c>
+      <c r="C241" t="str" s="7">
+        <v>Advisory Board member</v>
+      </c>
+      <c r="D241" t="str" s="7">
+        <v>present (start date unknown)</v>
+      </c>
+      <c r="E241" t="str" s="7">
+        <v>Maastricht University</v>
+      </c>
+      <c r="F241" t="str" s="7">
+        <v>High</v>
+      </c>
+      <c r="G241" t="str" s="7">
+        <v>https://ijmm.world/ijmm/advisory_board (verified 2026-10-13)</v>
+      </c>
+      <c r="H241" s="7"/>
+    </row>
+    <row r="242" ht="26.399999618530273" hidden="0" customHeight="1">
+      <c r="A242" t="str" s="7">
+        <v>International Journal of Music Mediation (IJMM)</v>
+      </c>
+      <c r="B242" t="str" s="7">
+        <v>Rineke Smilde</v>
+      </c>
+      <c r="C242" t="str" s="7">
+        <v>Advisory Board member</v>
+      </c>
+      <c r="D242" t="str" s="7">
+        <v>present (start date unknown)</v>
+      </c>
+      <c r="E242" t="str" s="7">
+        <v>Hanze University of Applied Sciences Groningen</v>
+      </c>
+      <c r="F242" t="str" s="7">
+        <v>High</v>
+      </c>
+      <c r="G242" t="str" s="7">
+        <v>https://ijmm.world/ijmm/advisory_board (verified 2026-10-13)</v>
+      </c>
+      <c r="H242" s="7"/>
+    </row>
+    <row r="243" ht="26.399999618530273" hidden="0" customHeight="1">
+      <c r="A243" t="str" s="7">
+        <v>International Journal of Music Mediation (IJMM)</v>
+      </c>
+      <c r="B243" t="str" s="7">
+        <v>Katja Thomson</v>
+      </c>
+      <c r="C243" t="str" s="7">
+        <v>Advisory Board member</v>
+      </c>
+      <c r="D243" t="str" s="7">
+        <v>present (start date unknown)</v>
+      </c>
+      <c r="E243" t="str" s="7">
+        <v>Sibelius Academy Helsinki</v>
+      </c>
+      <c r="F243" t="str" s="7">
+        <v>High</v>
+      </c>
+      <c r="G243" t="str" s="7">
+        <v>https://ijmm.world/ijmm/advisory_board (verified 2026-10-13)</v>
+      </c>
+      <c r="H243" s="7"/>
+    </row>
+    <row r="244" ht="26.399999618530273" hidden="0" customHeight="1">
+      <c r="A244" t="str" s="7">
+        <v>International Journal of Music Mediation (IJMM)</v>
+      </c>
+      <c r="B244" t="str" s="7">
+        <v>Jutta Toelle</v>
+      </c>
+      <c r="C244" t="str" s="7">
+        <v>Advisory Board member</v>
+      </c>
+      <c r="D244" t="str" s="7">
+        <v>present (start date unknown)</v>
+      </c>
+      <c r="E244" t="str" s="7">
+        <v>University of Music and Theatre Hamburg</v>
+      </c>
+      <c r="F244" t="str" s="7">
+        <v>High</v>
+      </c>
+      <c r="G244" t="str" s="7">
+        <v>https://ijmm.world/ijmm/advisory_board (verified 2026-10-13)</v>
+      </c>
+      <c r="H244" s="7"/>
+    </row>
+    <row r="245" ht="26.399999618530273" hidden="0" customHeight="1">
+      <c r="A245" t="str" s="7">
+        <v>International Journal of Music Mediation (IJMM)</v>
+      </c>
+      <c r="B245" t="str" s="7">
+        <v>Maria Westvall</v>
+      </c>
+      <c r="C245" t="str" s="7">
+        <v>Advisory Board member</v>
+      </c>
+      <c r="D245" t="str" s="7">
+        <v>present (start date unknown)</v>
+      </c>
+      <c r="E245" t="str" s="7">
+        <v>University College of Music Education Stockholm</v>
+      </c>
+      <c r="F245" t="str" s="7">
+        <v>High</v>
+      </c>
+      <c r="G245" t="str" s="7">
+        <v>https://ijmm.world/ijmm/advisory_board (verified 2026-10-13)</v>
+      </c>
+      <c r="H245" s="7"/>
+    </row>
+    <row r="246" ht="26.399999618530273" hidden="0" customHeight="1">
+      <c r="A246" t="str" s="7">
+        <v>International Journal of Music Mediation (IJMM)</v>
+      </c>
+      <c r="B246" t="str" s="7">
+        <v>Natasha Zielazinski</v>
+      </c>
+      <c r="C246" t="str" s="7">
+        <v>Advisory Board member</v>
+      </c>
+      <c r="D246" t="str" s="7">
+        <v>present (start date unknown)</v>
+      </c>
+      <c r="E246" t="str" s="7">
+        <v>Guildhall School of Music and Drama London</v>
+      </c>
+      <c r="F246" t="str" s="7">
+        <v>High</v>
+      </c>
+      <c r="G246" t="str" s="7">
+        <v>https://ijmm.world/ijmm/advisory_board (verified 2026-10-13)</v>
+      </c>
+      <c r="H246" s="7"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:H213"/>

</xml_diff>